<commit_message>
Add booking safeguards: DG advisories, pallet plan, price disclaimer
- Possible dangerous goods outside R-06: 21-entry ADR class 1-9 keyword
  catalogue (UN numbers checked against ADR 2025 Table A), safe-phrase
  filter, one Advisory per item; never changes Red/Amber/Green
- R-06 keywords: methanol added to flammable liquids; plain "tablets" and
  "fuel tablets" no longer trigger R-06
- Pallet plan by weight per carrier (min pallets, kg per pallet, cost,
  carton split) with click-to-apply buttons and a fewer-pallets Advisory
- Indicative price disclaimer on report, rate card and first chat price
- "Dates checked against today" line; duplicate Booking ID key trimmed
- Sample workbook: TB-21..TB-25 planted bookings; coverage matrix
- OpenSpec change add-booking-safeguards (15/15 tasks)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011k86CfG6sjkL5oopBdA73S
</commit_message>
<xml_diff>
--- a/assets/Preflight_Test_Cases.xlsx
+++ b/assets/Preflight_Test_Cases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expected results" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carrier options" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rulebook" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Allowed values" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field guide" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossary" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Bookings" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Items" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Expected results" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Carrier options" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Rulebook" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Allowed values" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Field guide" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Glossary" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32,6 +32,12 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF375623"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <i val="1"/>
       <color rgb="FF595959"/>
       <sz val="9"/>
@@ -43,18 +49,12 @@
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="FF375623"/>
-      <sz val="9"/>
+      <color theme="1"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
       <color rgb="FF595959"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color theme="1"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -103,14 +103,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor rgb="FFF2F2F2"/>
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE2EFDA"/>
-        <bgColor rgb="FFE2EFDA"/>
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -178,18 +178,18 @@
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -510,153 +510,153 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Bookings — one row per record. Row 3 is an example (grey); enter data from row 4.</t>
         </is>
       </c>
     </row>
     <row r="2" ht="31.5" customHeight="1" s="11">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Booking ID</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Seller name</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Origin city</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Origin country</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Destination city</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Destination country</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Destination type</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Ready to ship date</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Seller priority</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>Pallets</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>Cartons</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>Total declared value</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>Currency</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>Total gross weight (kg)</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>Delivery appointment booked</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>BK-001</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Northfield Goods</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Manchester</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>Frankfurt</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Warehouse</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>05-11-2026</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>Cheapest</t>
         </is>
       </c>
-      <c r="J3" s="4" t="n">
+      <c r="J3" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="K3" s="4" t="n">
+      <c r="K3" s="5" t="n">
         <v>90</v>
       </c>
-      <c r="L3" s="4" t="n">
+      <c r="L3" s="5" t="n">
         <v>5400</v>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="M3" s="5" t="inlineStr">
         <is>
           <t>GBP</t>
         </is>
       </c>
-      <c r="N3" s="4" t="n">
+      <c r="N3" s="5" t="n">
         <v>620</v>
       </c>
-      <c r="O3" s="4" t="inlineStr">
+      <c r="O3" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2041,54 +2041,349 @@
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="11">
-      <c r="C24" s="6" t="n"/>
-      <c r="D24" s="6" t="n"/>
-      <c r="E24" s="6" t="n"/>
-      <c r="F24" s="6" t="n"/>
-      <c r="G24" s="6" t="n"/>
-      <c r="I24" s="6" t="n"/>
-      <c r="M24" s="6" t="n"/>
-      <c r="O24" s="6" t="n"/>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>TB-21</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Confetti &amp; Co</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Business address</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>19-11-2026</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>Cheapest</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>1</v>
+      </c>
+      <c r="K24" t="n">
+        <v>20</v>
+      </c>
+      <c r="L24" t="n">
+        <v>1600</v>
+      </c>
+      <c r="M24" s="6" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>150</v>
+      </c>
+      <c r="O24" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="11">
-      <c r="C25" s="6" t="n"/>
-      <c r="D25" s="6" t="n"/>
-      <c r="E25" s="6" t="n"/>
-      <c r="F25" s="6" t="n"/>
-      <c r="G25" s="6" t="n"/>
-      <c r="I25" s="6" t="n"/>
-      <c r="M25" s="6" t="n"/>
-      <c r="O25" s="6" t="n"/>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>TB-22</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Blue Lagoon Pools</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Birmingham</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Business address</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>20-11-2026</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>Cheapest</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>2</v>
+      </c>
+      <c r="K25" t="n">
+        <v>25</v>
+      </c>
+      <c r="L25" t="n">
+        <v>3000</v>
+      </c>
+      <c r="M25" s="6" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>600</v>
+      </c>
+      <c r="O25" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="11">
-      <c r="C26" s="6" t="n"/>
-      <c r="D26" s="6" t="n"/>
-      <c r="E26" s="6" t="n"/>
-      <c r="F26" s="6" t="n"/>
-      <c r="G26" s="6" t="n"/>
-      <c r="I26" s="6" t="n"/>
-      <c r="M26" s="6" t="n"/>
-      <c r="O26" s="6" t="n"/>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TB-23</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Toolbox Toys</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Leeds</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>Business address</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>18-11-2026</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>Cheapest</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>1</v>
+      </c>
+      <c r="K26" t="n">
+        <v>30</v>
+      </c>
+      <c r="L26" t="n">
+        <v>2400</v>
+      </c>
+      <c r="M26" s="6" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
+        <v>200</v>
+      </c>
+      <c r="O26" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="11">
-      <c r="C27" s="6" t="n"/>
-      <c r="D27" s="6" t="n"/>
-      <c r="E27" s="6" t="n"/>
-      <c r="F27" s="6" t="n"/>
-      <c r="G27" s="6" t="n"/>
-      <c r="I27" s="6" t="n"/>
-      <c r="M27" s="6" t="n"/>
-      <c r="O27" s="6" t="n"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TB-24</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Loom &amp; Larder</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>Lyon</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Business address</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>19-11-2026</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>Cheapest</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>4</v>
+      </c>
+      <c r="K27" t="n">
+        <v>40</v>
+      </c>
+      <c r="L27" t="n">
+        <v>4000</v>
+      </c>
+      <c r="M27" s="6" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
+        <v>600</v>
+      </c>
+      <c r="O27" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="11">
-      <c r="C28" s="6" t="n"/>
-      <c r="D28" s="6" t="n"/>
-      <c r="E28" s="6" t="n"/>
-      <c r="F28" s="6" t="n"/>
-      <c r="G28" s="6" t="n"/>
-      <c r="I28" s="6" t="n"/>
-      <c r="M28" s="6" t="n"/>
-      <c r="O28" s="6" t="n"/>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> tb-05 </t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Alder Home</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>Warehouse</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>23-11-2026</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>Most reliable</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>1</v>
+      </c>
+      <c r="K28" t="n">
+        <v>10</v>
+      </c>
+      <c r="L28" t="n">
+        <v>900</v>
+      </c>
+      <c r="M28" s="6" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="N28" t="n">
+        <v>120</v>
+      </c>
+      <c r="O28" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="11">
       <c r="C29" s="6" t="n"/>
@@ -7364,99 +7659,99 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Items — one row per record. Row 3 is an example (grey); enter data from row 4.</t>
         </is>
       </c>
     </row>
     <row r="2" ht="31.5" customHeight="1" s="11">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Booking ID</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>SKU</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>HS code</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Quantity (units)</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Unit price</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Units per carton</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Cartons</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Unit weight (kg)</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>Country of origin</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>BK-001</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>MUG-01</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Ceramic coffee mug, 350 ml</t>
         </is>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="5" t="n">
         <v>691200</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" s="5" t="n">
         <v>1080</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="F3" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="G3" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="H3" s="5" t="n">
         <v>90</v>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="I3" s="5" t="n">
         <v>0.5</v>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
@@ -8495,57 +8790,242 @@
     <row r="30" ht="15.75" customHeight="1" s="11">
       <c r="A30" t="inlineStr">
         <is>
-          <t>TB-99</t>
+          <t>TB-21</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>GHOST-01</t>
+          <t>PP-01</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Item pointing at a booking that does not exist</t>
+          <t>Party poppers, box of 50</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>691200</v>
+        <v>950590</v>
       </c>
       <c r="E30" t="n">
-        <v>10</v>
+        <v>200</v>
       </c>
       <c r="F30" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G30" t="n">
         <v>10</v>
       </c>
       <c r="H30" t="n">
+        <v>20</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J30" s="6" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15.75" customHeight="1" s="11">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>TB-22</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>CHL-01</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Pool chlorine granules 5 kg tub</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>380894</v>
+      </c>
+      <c r="E31" t="n">
+        <v>100</v>
+      </c>
+      <c r="F31" t="n">
+        <v>30</v>
+      </c>
+      <c r="G31" t="n">
+        <v>4</v>
+      </c>
+      <c r="H31" t="n">
+        <v>25</v>
+      </c>
+      <c r="I31" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="J31" s="6" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15.75" customHeight="1" s="11">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>TB-23</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>SL-01</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Spirit level 60 cm</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>901580</v>
+      </c>
+      <c r="E32" t="n">
+        <v>100</v>
+      </c>
+      <c r="F32" t="n">
+        <v>12</v>
+      </c>
+      <c r="G32" t="n">
+        <v>10</v>
+      </c>
+      <c r="H32" t="n">
+        <v>10</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="15.75" customHeight="1" s="11">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>TB-23</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>MC-01</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Matchbox car set</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>950300</v>
+      </c>
+      <c r="E33" t="n">
+        <v>200</v>
+      </c>
+      <c r="F33" t="n">
+        <v>6</v>
+      </c>
+      <c r="G33" t="n">
+        <v>10</v>
+      </c>
+      <c r="H33" t="n">
+        <v>20</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="15.75" customHeight="1" s="11">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>TB-24</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>BLK-01</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Wool blanket, double</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>630120</v>
+      </c>
+      <c r="E34" t="n">
+        <v>200</v>
+      </c>
+      <c r="F34" t="n">
+        <v>20</v>
+      </c>
+      <c r="G34" t="n">
+        <v>5</v>
+      </c>
+      <c r="H34" t="n">
+        <v>40</v>
+      </c>
+      <c r="I34" t="n">
+        <v>2</v>
+      </c>
+      <c r="J34" s="6" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="15.75" customHeight="1" s="11">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>TB-99</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>GHOST-01</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Item pointing at a booking that does not exist</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>691200</v>
+      </c>
+      <c r="E35" t="n">
+        <v>10</v>
+      </c>
+      <c r="F35" t="n">
         <v>1</v>
       </c>
-      <c r="I30" t="n">
+      <c r="G35" t="n">
+        <v>10</v>
+      </c>
+      <c r="H35" t="n">
+        <v>1</v>
+      </c>
+      <c r="I35" t="n">
         <v>0.5</v>
       </c>
-      <c r="J30" s="6" t="inlineStr">
+      <c r="J35" s="6" t="inlineStr">
         <is>
           <t>China</t>
         </is>
       </c>
-    </row>
-    <row r="31" ht="15.75" customHeight="1" s="11">
-      <c r="J31" s="6" t="n"/>
-    </row>
-    <row r="32" ht="15.75" customHeight="1" s="11">
-      <c r="J32" s="6" t="n"/>
-    </row>
-    <row r="33" ht="15.75" customHeight="1" s="11">
-      <c r="J33" s="6" t="n"/>
-    </row>
-    <row r="34" ht="15.75" customHeight="1" s="11">
-      <c r="J34" s="6" t="n"/>
-    </row>
-    <row r="35" ht="15.75" customHeight="1" s="11">
-      <c r="J35" s="6" t="n"/>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="11">
       <c r="J36" s="6" t="n"/>
@@ -10459,7 +10939,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="11" min="1" max="1"/>
@@ -10472,7 +10952,7 @@
     <row r="1">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>Test cases — what Preflight should report for each booking above (checked on or before 16-11-2026; after that, every date becomes “past” and R-10 fires).</t>
+          <t>Test cases — what Preflight should report for each booking above (advisories never change the status) (checked on or before 16-11-2026; after that, every date becomes “past” and R-10 fires).</t>
         </is>
       </c>
     </row>
@@ -11046,25 +11526,160 @@
     <row r="23">
       <c r="A23" s="16" t="inlineStr">
         <is>
+          <t>TB-21</t>
+        </is>
+      </c>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>Party poppers — ADR class 1 (fireworks), outside the R-06 categories</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>— (Advisory: possible dangerous goods, ADR class 1)</t>
+        </is>
+      </c>
+      <c r="E23" s="16" t="inlineStr">
+        <is>
+          <t>Carrier A · Road economy (£170)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="inlineStr">
+        <is>
+          <t>TB-22</t>
+        </is>
+      </c>
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>Pool chlorine — ADR class 5.1 (oxidiser), outside the R-06 categories</t>
+        </is>
+      </c>
+      <c r="C24" s="17" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>— (Advisory: possible dangerous goods, ADR class 5.1)</t>
+        </is>
+      </c>
+      <c r="E24" s="16" t="inlineStr">
+        <is>
+          <t>Carrier A · Road economy (£320)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>TB-23</t>
+        </is>
+      </c>
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>Look-alike words: “spirit level” and “matchbox car” are not dangerous goods</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="16" t="inlineStr">
+        <is>
+          <t>Carrier A · Road economy (£180)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>TB-24</t>
+        </is>
+      </c>
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>600 kg on 4 pallets — 2 pallets are enough by weight</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="D26" s="16" t="inlineStr">
+        <is>
+          <t>— (Advisory: 2 pallets enough, saving £340)</t>
+        </is>
+      </c>
+      <c r="E26" s="16" t="inlineStr">
+        <is>
+          <t>Carrier A · Road economy (£680)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> tb-05 </t>
+        </is>
+      </c>
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>Booking ID “ tb-05 ” repeats TB-05 (different case and spaces)</t>
+        </is>
+      </c>
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>Data: duplicate Booking ID (its items cannot be matched)</t>
+        </is>
+      </c>
+      <c r="E27" s="16" t="inlineStr">
+        <is>
+          <t>Carrier C · Road express (£340)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
           <t>TB-99 (Items only)</t>
         </is>
       </c>
-      <c r="B23" s="16" t="inlineStr">
+      <c r="B28" s="16" t="inlineStr">
         <is>
           <t>Item row whose Booking ID is not on the Bookings sheet</t>
         </is>
       </c>
-      <c r="C23" s="20" t="inlineStr">
+      <c r="C28" s="20" t="inlineStr">
         <is>
           <t>Notice</t>
         </is>
       </c>
-      <c r="D23" s="16" t="inlineStr">
+      <c r="D28" s="16" t="inlineStr">
         <is>
           <t>Reported as an orphan item row, not checked</t>
         </is>
       </c>
-      <c r="E23" s="16" t="inlineStr">
+      <c r="E28" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -11096,407 +11711,407 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>FIXED - judges will use exactly this rate card. Do not edit.</t>
         </is>
       </c>
     </row>
     <row r="2" ht="31.5" customHeight="1" s="11">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Carrier</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Service</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Origin country</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Destination country</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Price per pallet</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Currency</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Transit time (days)</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>On-time rate (%)</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Max weight per pallet (kg)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Carrier A</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Road economy</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="E3" s="5" t="n">
+      <c r="E3" s="4" t="n">
         <v>180</v>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>GBP</t>
         </is>
       </c>
-      <c r="G3" s="5" t="n">
+      <c r="G3" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="H3" s="5" t="n">
+      <c r="H3" s="4" t="n">
         <v>92</v>
       </c>
-      <c r="I3" s="5" t="n">
+      <c r="I3" s="4" t="n">
         <v>500</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Carrier B</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Road standard</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="E4" s="5" t="n">
+      <c r="E4" s="4" t="n">
         <v>220</v>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>GBP</t>
         </is>
       </c>
-      <c r="G4" s="5" t="n">
+      <c r="G4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H4" s="5" t="n">
+      <c r="H4" s="4" t="n">
         <v>95</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="I4" s="4" t="n">
         <v>750</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Carrier C</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Road express</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="4" t="n">
         <v>340</v>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>GBP</t>
         </is>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="G5" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="H5" s="4" t="n">
         <v>98</v>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="I5" s="4" t="n">
         <v>400</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Carrier A</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Road economy</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="4" t="n">
         <v>170</v>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>GBP</t>
         </is>
       </c>
-      <c r="G6" s="5" t="n">
+      <c r="G6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="H6" s="4" t="n">
         <v>92</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="I6" s="4" t="n">
         <v>500</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Carrier B</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Road standard</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="4" t="n">
         <v>210</v>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>GBP</t>
         </is>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="G7" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="H7" s="4" t="n">
         <v>95</v>
       </c>
-      <c r="I7" s="5" t="n">
+      <c r="I7" s="4" t="n">
         <v>750</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Carrier C</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Road express</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="4" t="n">
         <v>330</v>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>GBP</t>
         </is>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="G8" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="H8" s="4" t="n">
         <v>98</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="I8" s="4" t="n">
         <v>400</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Carrier A</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Road economy</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Netherlands</t>
         </is>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="4" t="n">
         <v>160</v>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>GBP</t>
         </is>
       </c>
-      <c r="G9" s="5" t="n">
+      <c r="G9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="H9" s="4" t="n">
         <v>92</v>
       </c>
-      <c r="I9" s="5" t="n">
+      <c r="I9" s="4" t="n">
         <v>500</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Carrier B</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Road standard</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Netherlands</t>
         </is>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" s="4" t="n">
         <v>200</v>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>GBP</t>
         </is>
       </c>
-      <c r="G10" s="5" t="n">
+      <c r="G10" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="H10" s="4" t="n">
         <v>95</v>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="I10" s="4" t="n">
         <v>750</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Carrier C</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Road express</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Netherlands</t>
         </is>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="E11" s="4" t="n">
         <v>320</v>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>GBP</t>
         </is>
       </c>
-      <c r="G11" s="5" t="n">
+      <c r="G11" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H11" s="5" t="n">
+      <c r="H11" s="4" t="n">
         <v>98</v>
       </c>
-      <c r="I11" s="5" t="n">
+      <c r="I11" s="4" t="n">
         <v>400</v>
       </c>
     </row>
@@ -12502,194 +13117,194 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>FIXED - these are the only rules judges will test against. Do not edit.</t>
         </is>
       </c>
     </row>
     <row r="2" ht="31.5" customHeight="1" s="11">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Rule ID</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Rule</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Severity if broken</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>R-01</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Every item must have an HS code of at least 6 digits</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>R-02</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Total declared value must equal the sum of quantity × unit price across all items (within 1%)</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>R-03</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>For each item, units per carton × cartons must equal quantity</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>R-04</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Total cartons on the booking must equal the sum of cartons across all items</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>R-05</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Weight per pallet (total gross weight ÷ pallets) must not exceed the chosen carrier's max weight per pallet</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>R-06</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>No lithium batteries, aerosols or flammable liquids</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>R-07</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Total gross weight must be at least the sum of unit weight × quantity across all items</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Amber</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>R-08</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Shipments to a warehouse must have a delivery appointment booked</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Amber</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>R-09</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Every item must have a country of origin</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Amber</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>R-10</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Ready to ship date must not be in the past</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Amber</t>
         </is>

</xml_diff>